<commit_message>
add 4node and 6node
</commit_message>
<xml_diff>
--- a/4node_spain/output_all.xlsx
+++ b/4node_spain/output_all.xlsx
@@ -447,16 +447,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8.870336419705509e-06</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1.328016901018055</v>
+        <v>1.338411277415557</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5144481827776213</v>
+        <v>0.003052137218589517</v>
       </c>
       <c r="D2" t="n">
-        <v>1.178377716999204</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -505,13 +505,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1.724404365356792e-05</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>9.871345059498339e-07</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>7.033013450984647e-07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -521,16 +521,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.724404365356792e-05</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1.974535298499556e-06</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2.213103850403893</v>
+        <v>2.230685462359261</v>
       </c>
     </row>
     <row r="4">
@@ -540,16 +540,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.871345059498339e-07</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1.974535298499556e-06</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8572568171758366</v>
+        <v>0.005086895364315862</v>
       </c>
     </row>
     <row r="5">
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.033013450984647e-07</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>2.213103850403893</v>
+        <v>2.230685462359261</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8572568171758366</v>
+        <v>0.005086895364315862</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -614,16 +614,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>8.578384587121235e-07</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>3.838004580813958e-09</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>1.624558509938367e-08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -633,16 +633,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8.76107205227683e-07</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>7.005976243590339e-09</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2331570933881284</v>
+        <v>0.235009558063097</v>
       </c>
     </row>
     <row r="4">
@@ -652,16 +652,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.636549362693529e-08</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>3.75040287714512e-09</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2392515214723587</v>
+        <v>0.001419700923970157</v>
       </c>
     </row>
     <row r="5">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.533191484881513e-08</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2307501695627795</v>
+        <v>0.2325833650998232</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2371914917096857</v>
+        <v>0.001407476612128359</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -729,13 +729,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9999991421615413</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9999999961619954</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9999999837544149</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -745,16 +745,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9999991238927948</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9999999929940238</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7668429066118716</v>
+        <v>0.764990441936903</v>
       </c>
     </row>
     <row r="4">
@@ -764,16 +764,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9999999836345064</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9999999962495971</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7607484785276413</v>
+        <v>0.9985802990760299</v>
       </c>
     </row>
     <row r="5">
@@ -783,13 +783,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9999999846680852</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7692498304372205</v>
+        <v>0.7674166349001768</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7628085082903143</v>
+        <v>0.9985925233878716</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -851,13 +851,13 @@
         <v/>
       </c>
       <c r="E2" t="n">
-        <v>8.641737665572962e-07</v>
+        <v/>
       </c>
       <c r="F2" t="n">
-        <v>1.571886043866166e-09</v>
+        <v/>
       </c>
       <c r="G2" t="n">
-        <v>1.038849272633128e-09</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -880,13 +880,13 @@
         <v/>
       </c>
       <c r="E3" t="n">
-        <v>-6.039083291940105e-11</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1.426354460357299e-08</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>7.644016581504995e-10</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -897,7 +897,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.001</v>
+        <v/>
       </c>
       <c r="E4" t="n">
-        <v>1.341956427971047e-09</v>
+        <v/>
       </c>
       <c r="F4" t="n">
-        <v>1.364058044834568e-09</v>
+        <v/>
       </c>
       <c r="G4" t="n">
-        <v>1.42182330644189e-08</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -926,25 +926,25 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>-6.628894407890576e-10</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>5.498739941837663e-11</v>
+        <v/>
       </c>
       <c r="G5" t="n">
-        <v>2.484879310713614e-10</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -955,36 +955,36 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>-1.187599329040472e-09</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>1.090707115058811e-09</v>
+        <v/>
       </c>
       <c r="G6" t="n">
-        <v>1.481800818731853e-10</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -996,24 +996,24 @@
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>-1.29516104229539e-09</v>
+        <v/>
       </c>
       <c r="F7" t="n">
-        <v>-6.410771496789424e-10</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>3.279253925303872e-12</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1022,51 +1022,51 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.001</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>-4.013377055928725e-10</v>
+        <v/>
       </c>
       <c r="F8" t="n">
-        <v>-5.076274639924246e-10</v>
+        <v/>
       </c>
       <c r="G8" t="n">
-        <v>6.399653150345989e-11</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>-8.009057933067289e-10</v>
+        <v/>
       </c>
       <c r="F9" t="n">
-        <v>-5.257085988851518e-10</v>
+        <v/>
       </c>
       <c r="G9" t="n">
-        <v>1.069841545724073e-10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1080,22 +1080,22 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>-1.250759887063155e-09</v>
+        <v/>
       </c>
       <c r="F10" t="n">
-        <v>-8.256304863162183e-10</v>
+        <v/>
       </c>
       <c r="G10" t="n">
-        <v>1.656723186418905e-11</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1112,19 +1112,19 @@
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>1.064227859300096e-09</v>
+        <v/>
       </c>
       <c r="F11" t="n">
-        <v>4.526399873981312e-10</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>-3.124844514587847e-10</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1134,234 +1134,234 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>-1.0631791366334e-09</v>
+        <v/>
       </c>
       <c r="F12" t="n">
-        <v>-5.415600802491707e-10</v>
+        <v/>
       </c>
       <c r="G12" t="n">
-        <v>-7.458861603338213e-10</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>i4</t>
+          <t>i1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.001</v>
+        <v/>
       </c>
       <c r="E13" t="n">
-        <v>-1.205013224026331e-09</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>-1.37294983188906e-11</v>
+        <v/>
       </c>
       <c r="G13" t="n">
-        <v>-7.250338221020084e-10</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i1</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-1.216031440211161e-09</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
         <v/>
       </c>
       <c r="F14" t="n">
-        <v>-2.185302127329404e-11</v>
+        <v/>
       </c>
       <c r="G14" t="n">
-        <v>-4.572289951267954e-10</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-1.386707643015959e-09</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
         <v/>
       </c>
       <c r="F15" t="n">
-        <v>-5.80790425285323e-11</v>
+        <v/>
       </c>
       <c r="G15" t="n">
-        <v>-9.916829304342753e-10</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>i4</t>
+          <t>i1</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-1.362524264787633e-09</v>
+        <v/>
       </c>
       <c r="E16" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>-2.381728241959801e-10</v>
+        <v/>
       </c>
       <c r="G16" t="n">
-        <v>9.849625178174854e-11</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8.731021938324944e-07</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v/>
       </c>
       <c r="F17" t="n">
-        <v>5.031549108791214e-10</v>
+        <v/>
       </c>
       <c r="G17" t="n">
-        <v>6.114709127771406e-10</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.725025260226002e-09</v>
+        <v/>
       </c>
       <c r="E18" t="n">
         <v/>
       </c>
       <c r="F18" t="n">
-        <v>7.522518961960364e-09</v>
+        <v/>
       </c>
       <c r="G18" t="n">
-        <v>2.545622285000044e-09</v>
+        <v>0.9999999999999993</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>i4</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>-7.814616246460973e-10</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>0.001</v>
+        <v/>
       </c>
       <c r="F19" t="n">
-        <v>4.373171321700525e-10</v>
+        <v/>
       </c>
       <c r="G19" t="n">
-        <v>0.233157106089259</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1370,22 +1370,22 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>-1.020121398075272e-09</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v/>
       </c>
       <c r="F20" t="n">
-        <v>-5.850390127279153e-10</v>
+        <v/>
       </c>
       <c r="G20" t="n">
-        <v>-8.552232824431467e-10</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1399,51 +1399,51 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2.319493393601922e-09</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>0.001</v>
+        <v/>
       </c>
       <c r="F21" t="n">
-        <v>1.539533263130401e-10</v>
+        <v/>
       </c>
       <c r="G21" t="n">
-        <v>1.528677164356876e-09</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>i4</t>
+          <t>i2</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-1.238291546764599e-09</v>
+        <v/>
       </c>
       <c r="E22" t="n">
-        <v/>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>-5.855288502619328e-10</v>
+        <v/>
       </c>
       <c r="G22" t="n">
-        <v>-3.162072656368193e-10</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>i2</t>
+          <t>i4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1453,20 +1453,20 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>i1</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-1.001578734659124e-09</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v/>
       </c>
       <c r="F23" t="n">
-        <v>-2.362207861187677e-10</v>
+        <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.106663304087873e-09</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1486,16 +1486,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>-1.103461533040981e-09</v>
-      </c>
-      <c r="E24" t="n">
-        <v/>
+        <v>-4.521193438935204e-13</v>
       </c>
       <c r="F24" t="n">
-        <v>-1.321003748246094e-10</v>
+        <v>-9.218898292635228e-14</v>
       </c>
       <c r="G24" t="n">
-        <v>-1.069684738707974e-09</v>
+        <v>-9.213319273692388e-15</v>
       </c>
     </row>
     <row r="25">
@@ -1515,16 +1512,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>-1.277237168500421e-09</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.001</v>
+        <v>-4.896970774049776e-13</v>
       </c>
       <c r="F25" t="n">
-        <v>-1.806338119189837e-11</v>
+        <v>-3.974669676310409e-14</v>
       </c>
       <c r="G25" t="n">
-        <v>-1.196692738104964e-09</v>
+        <v>9.443835975480529e-12</v>
       </c>
     </row>
     <row r="26">
@@ -1544,16 +1538,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-8.39435753469942e-10</v>
+        <v>-2.461620825430208e-13</v>
       </c>
       <c r="E26" t="n">
-        <v>-3.299697886362185e-12</v>
-      </c>
-      <c r="F26" t="n">
-        <v/>
+        <v>7.158761416609687e-14</v>
       </c>
       <c r="G26" t="n">
-        <v>5.078387276867497e-09</v>
+        <v>4.946083732873077e-11</v>
       </c>
     </row>
     <row r="27">
@@ -1573,16 +1564,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-7.100582984279928e-10</v>
+        <v>-1.989516352314706e-13</v>
       </c>
       <c r="E27" t="n">
-        <v>-1.323442078789982e-10</v>
-      </c>
-      <c r="F27" t="n">
-        <v/>
+        <v>2.53628056543727e-15</v>
       </c>
       <c r="G27" t="n">
-        <v>-1.6738462563871e-11</v>
+        <v>1.441188173816939e-15</v>
       </c>
     </row>
     <row r="28">
@@ -1602,16 +1590,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-7.477538669636364e-10</v>
+        <v>-2.074593122945222e-13</v>
       </c>
       <c r="E28" t="n">
-        <v>-2.59947487905265e-10</v>
-      </c>
-      <c r="F28" t="n">
-        <v/>
+        <v>-2.252777828781662e-14</v>
       </c>
       <c r="G28" t="n">
-        <v>2.07210881930879e-08</v>
+        <v>2.022396438118486e-10</v>
       </c>
     </row>
     <row r="29">
@@ -1631,16 +1616,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>7.646712353245158e-10</v>
+        <v>3.129094204961878e-13</v>
       </c>
       <c r="E29" t="n">
-        <v>-5.00178886442195e-10</v>
-      </c>
-      <c r="F29" t="n">
-        <v/>
+        <v>-1.226048659437124e-13</v>
       </c>
       <c r="G29" t="n">
-        <v>8.146005403432506e-09</v>
+        <v>8.348183734364837e-11</v>
       </c>
     </row>
     <row r="30">
@@ -1660,16 +1642,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.013817141593131e-09</v>
+        <v>3.347254331708843e-13</v>
       </c>
       <c r="E30" t="n">
-        <v>2.128528854518318e-10</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0.001</v>
+        <v>6.863537964128549e-14</v>
       </c>
       <c r="G30" t="n">
-        <v>2.329606419331658e-10</v>
+        <v>4.234349534632272e-15</v>
       </c>
     </row>
     <row r="31">
@@ -1689,16 +1668,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>-4.092658771091214e-10</v>
+        <v>-1.477936841667924e-13</v>
       </c>
       <c r="E31" t="n">
-        <v>-5.588248940072951e-10</v>
-      </c>
-      <c r="F31" t="n">
-        <v/>
+        <v>-1.919370813573443e-13</v>
       </c>
       <c r="G31" t="n">
-        <v>1.931443523368534e-08</v>
+        <v>1.580446582257884e-10</v>
       </c>
     </row>
     <row r="32">
@@ -1718,16 +1694,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.446793726010728e-08</v>
+        <v>4.79731133804684e-12</v>
       </c>
       <c r="E32" t="n">
-        <v>3.349855677523292e-10</v>
-      </c>
-      <c r="F32" t="n">
-        <v/>
+        <v>1.941235812106928e-13</v>
       </c>
       <c r="G32" t="n">
-        <v>1.410386107969743e-08</v>
+        <v>1.3059618036051e-10</v>
       </c>
     </row>
     <row r="33">
@@ -1747,16 +1720,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2.852861299503332e-09</v>
+        <v>9.617449994470711e-13</v>
       </c>
       <c r="E33" t="n">
-        <v>7.596075338345244e-09</v>
-      </c>
-      <c r="F33" t="n">
-        <v/>
+        <v>2.297140483531683e-12</v>
       </c>
       <c r="G33" t="n">
-        <v>2.01730394716494e-08</v>
+        <v>1.634697593975356e-10</v>
       </c>
     </row>
     <row r="34">
@@ -1776,16 +1746,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6.892179922648861e-10</v>
+        <v>1.866594849443035e-13</v>
       </c>
       <c r="E34" t="n">
-        <v>4.193240418619008e-10</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0.001</v>
+        <v>6.55607475988589e-14</v>
       </c>
       <c r="G34" t="n">
-        <v>0.2392514783420213</v>
+        <v>0.2423384116817981</v>
       </c>
     </row>
     <row r="35">
@@ -1805,16 +1772,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4.80160192858192e-10</v>
+        <v>1.855957265000344e-13</v>
       </c>
       <c r="E35" t="n">
-        <v>-2.303980749739834e-10</v>
-      </c>
-      <c r="F35" t="n">
-        <v/>
+        <v>-1.815028850054462e-14</v>
       </c>
       <c r="G35" t="n">
-        <v>3.532870524268979e-09</v>
+        <v>3.762390462459224e-11</v>
       </c>
     </row>
     <row r="36">
@@ -1834,16 +1798,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>-6.442030463061184e-10</v>
+        <v>-2.214398085931662e-13</v>
       </c>
       <c r="E36" t="n">
-        <v>-8.854159275574385e-11</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0.001</v>
+        <v>-6.43365369581145e-14</v>
       </c>
       <c r="G36" t="n">
-        <v>2.4419745305257e-09</v>
+        <v>2.860013319270978e-11</v>
       </c>
     </row>
     <row r="37">
@@ -1863,16 +1824,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>-3.037588983350803e-10</v>
+        <v>-1.313845651555103e-13</v>
       </c>
       <c r="E37" t="n">
-        <v>-8.050867232058524e-11</v>
-      </c>
-      <c r="F37" t="n">
-        <v/>
+        <v>-6.736417892230797e-14</v>
       </c>
       <c r="G37" t="n">
-        <v>-2.160689054803325e-10</v>
+        <v>-3.204287821035392e-15</v>
       </c>
     </row>
     <row r="38">
@@ -1892,16 +1850,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-6.124159753753544e-10</v>
+        <v>-1.986873665234649e-13</v>
       </c>
       <c r="E38" t="n">
-        <v>-5.622343860346513e-10</v>
+        <v>5.435248773214e-11</v>
       </c>
       <c r="F38" t="n">
-        <v>7.361295014414699e-09</v>
-      </c>
-      <c r="G38" t="n">
-        <v/>
+        <v>7.357580182894461e-11</v>
       </c>
     </row>
     <row r="39">
@@ -1921,16 +1876,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-6.687951565510892e-10</v>
+        <v>-2.141843592904098e-13</v>
       </c>
       <c r="E39" t="n">
-        <v>-1.006210907862035e-09</v>
+        <v>2.447498330217321e-11</v>
       </c>
       <c r="F39" t="n">
-        <v>1.511083200562494e-08</v>
-      </c>
-      <c r="G39" t="n">
-        <v/>
+        <v>1.713009211183659e-10</v>
       </c>
     </row>
     <row r="40">
@@ -1950,16 +1902,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-3.223209985784286e-11</v>
+        <v>1.95385818142674e-14</v>
       </c>
       <c r="E40" t="n">
-        <v>1.527822557002831e-09</v>
+        <v>9.328812891341984e-15</v>
       </c>
       <c r="F40" t="n">
-        <v>1.568081057487282e-10</v>
-      </c>
-      <c r="G40" t="n">
-        <v/>
+        <v>3.79293940604435e-15</v>
       </c>
     </row>
     <row r="41">
@@ -1979,16 +1928,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>-1.027755583893186e-11</v>
+        <v>-1.148991823819693e-14</v>
       </c>
       <c r="E41" t="n">
-        <v>-1.191298439476066e-09</v>
+        <v>1.151523034985745e-11</v>
       </c>
       <c r="F41" t="n">
-        <v>4.401284402739772e-09</v>
-      </c>
-      <c r="G41" t="n">
-        <v/>
+        <v>5.197835200060393e-11</v>
       </c>
     </row>
     <row r="42">
@@ -2008,16 +1954,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-1.553391956397661e-11</v>
+        <v>-1.929329214540669e-15</v>
       </c>
       <c r="E42" t="n">
-        <v>-1.077987319569966e-09</v>
+        <v>1.599966859729875e-11</v>
       </c>
       <c r="F42" t="n">
-        <v>2.117691491368347e-08</v>
-      </c>
-      <c r="G42" t="n">
-        <v/>
+        <v>2.026898076120792e-10</v>
       </c>
     </row>
     <row r="43">
@@ -2037,16 +1980,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>-1.123717379950717e-11</v>
+        <v>-2.754055700073404e-14</v>
       </c>
       <c r="E43" t="n">
-        <v>-9.744376820817634e-10</v>
+        <v>-5.34022604209367e-15</v>
       </c>
       <c r="F43" t="n">
-        <v>3.416147476553469e-12</v>
-      </c>
-      <c r="G43" t="n">
-        <v/>
+        <v>8.729459670519887e-16</v>
       </c>
     </row>
     <row r="44">
@@ -2066,16 +2006,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>-1.239070526975528e-10</v>
+        <v>-3.986481792089907e-14</v>
       </c>
       <c r="E44" t="n">
-        <v>-1.103340225149276e-09</v>
+        <v>1.531537112019994e-11</v>
       </c>
       <c r="F44" t="n">
-        <v>2.556549242255614e-09</v>
-      </c>
-      <c r="G44" t="n">
-        <v/>
+        <v>3.601827345605835e-11</v>
       </c>
     </row>
     <row r="45">
@@ -2095,16 +2032,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2.546480673964905e-11</v>
+        <v>1.004910859197107e-14</v>
       </c>
       <c r="E45" t="n">
-        <v>-2.523954097028532e-10</v>
+        <v>7.283977002913996e-11</v>
       </c>
       <c r="F45" t="n">
-        <v>4.349930487942298e-09</v>
-      </c>
-      <c r="G45" t="n">
-        <v/>
+        <v>5.239349518019633e-11</v>
       </c>
     </row>
     <row r="46">
@@ -2124,16 +2058,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.346922094645803e-11</v>
+        <v>1.117681419140802e-14</v>
       </c>
       <c r="E46" t="n">
-        <v>-5.532138064137541e-10</v>
+        <v>2.334383741751352e-15</v>
       </c>
       <c r="F46" t="n">
-        <v>-1.595243384809146e-10</v>
-      </c>
-      <c r="G46" t="n">
-        <v/>
+        <v>-1.25668746261097e-15</v>
       </c>
     </row>
     <row r="47">
@@ -2153,16 +2084,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.295968730580179e-08</v>
+        <v>4.675327317877675e-12</v>
       </c>
       <c r="E47" t="n">
-        <v>2.254015927847025e-09</v>
+        <v>5.200619837714409e-11</v>
       </c>
       <c r="F47" t="n">
-        <v>1.567110148075361e-08</v>
-      </c>
-      <c r="G47" t="n">
-        <v/>
+        <v>1.568838904300618e-10</v>
       </c>
     </row>
     <row r="48">
@@ -2182,16 +2110,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>5.499025194344608e-10</v>
+        <v>1.485627475409073e-13</v>
       </c>
       <c r="E48" t="n">
-        <v>0.2307501713557361</v>
+        <v>0.230595612696682</v>
       </c>
       <c r="F48" t="n">
-        <v>1.387038996154108e-08</v>
-      </c>
-      <c r="G48" t="n">
-        <v/>
+        <v>1.286997355495077e-10</v>
       </c>
     </row>
     <row r="49">
@@ -2211,16 +2136,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6.2935605109449e-10</v>
+        <v>1.986229134569287e-13</v>
       </c>
       <c r="E49" t="n">
-        <v>1.752487860327088e-10</v>
+        <v>4.76828236336163e-11</v>
       </c>
       <c r="F49" t="n">
-        <v>0.2371914649215917</v>
-      </c>
-      <c r="G49" t="n">
-        <v/>
+        <v>0.2402517607222237</v>
       </c>
     </row>
   </sheetData>
@@ -2239,7 +2161,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>0.0075015</v>
+        <v>1.437000000005355</v>
       </c>
     </row>
   </sheetData>
@@ -2280,16 +2202,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3.223869379218018e-06</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1.91920451826095e-06</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1.118667332369326e-08</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6639954888086967</v>
+        <v>1.341463414634146</v>
       </c>
     </row>
   </sheetData>
@@ -2308,7 +2230,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>2.437860993662113e-15</v>
+        <v>1.387893989894815e-12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
6node and 4node with results except for 6MIP
</commit_message>
<xml_diff>
--- a/4node_spain/output_all.xlsx
+++ b/4node_spain/output_all.xlsx
@@ -450,13 +450,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.2497696519922655</v>
+        <v>0.6674723302746098</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4995392840625252</v>
+        <v>1.335005592754358</v>
       </c>
     </row>
   </sheetData>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8325655117677805</v>
+        <v>2.225009312414772</v>
       </c>
     </row>
     <row r="4">
@@ -562,7 +562,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8325655117677805</v>
+        <v>2.225009312414772</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08771333125067682</v>
+        <v>0.2344115578142438</v>
       </c>
     </row>
     <row r="4">
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.08680779863780597</v>
+        <v>0.2319915390806588</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -754,7 +754,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9122866687493232</v>
+        <v>0.7655884421857562</v>
       </c>
     </row>
     <row r="4">
@@ -786,7 +786,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0.913192201362194</v>
+        <v>0.7680084609193412</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -851,13 +851,13 @@
         <v/>
       </c>
       <c r="E2" t="n">
-        <v>7.536903440509053e-11</v>
+        <v>3.815739899730097e-10</v>
       </c>
       <c r="F2" t="n">
-        <v>2.530404361924982e-11</v>
+        <v>6.159100397583726e-13</v>
       </c>
       <c r="G2" t="n">
-        <v>2.829484303972412e-11</v>
+        <v>3.422889739670045e-13</v>
       </c>
     </row>
     <row r="3">
@@ -880,13 +880,13 @@
         <v/>
       </c>
       <c r="E3" t="n">
-        <v>2.177699981004078e-11</v>
+        <v>-1.256195458777838e-13</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.385508950076968e-11</v>
+        <v>3.760373443993653e-12</v>
       </c>
       <c r="G3" t="n">
-        <v>2.170386308648477e-11</v>
+        <v>2.67503656462772e-13</v>
       </c>
     </row>
     <row r="4">
@@ -909,13 +909,13 @@
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>4.998461880768954e-12</v>
+        <v>4.706214736577288e-13</v>
       </c>
       <c r="F4" t="n">
-        <v>6.021721063842069e-13</v>
+        <v>4.735704304002241e-13</v>
       </c>
       <c r="G4" t="n">
-        <v>-2.093667185917307e-11</v>
+        <v>4.809979311678474e-12</v>
       </c>
     </row>
     <row r="5">
@@ -938,13 +938,13 @@
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>-1.559599994926858e-12</v>
+        <v>-2.459467748884885e-13</v>
       </c>
       <c r="F5" t="n">
-        <v>8.286162495528272e-12</v>
+        <v>3.826524836120517e-14</v>
       </c>
       <c r="G5" t="n">
-        <v>3.845363970157252e-12</v>
+        <v>8.643970103117607e-14</v>
       </c>
     </row>
     <row r="6">
@@ -967,13 +967,13 @@
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>-1.231971509129084e-11</v>
+        <v>-4.388205997144859e-13</v>
       </c>
       <c r="F6" t="n">
-        <v>4.343236828506426e-12</v>
+        <v>5.045842221238413e-13</v>
       </c>
       <c r="G6" t="n">
-        <v>6.362446078474903e-13</v>
+        <v>6.630934018001609e-14</v>
       </c>
     </row>
     <row r="7">
@@ -996,13 +996,13 @@
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>2.355287122770818e-12</v>
+        <v>-4.676900047415983e-13</v>
       </c>
       <c r="F7" t="n">
-        <v>7.839662507537922e-12</v>
+        <v>-1.919543389263195e-13</v>
       </c>
       <c r="G7" t="n">
-        <v>1.974571748785166e-11</v>
+        <v>-5.675247778036226e-15</v>
       </c>
     </row>
     <row r="8">
@@ -1025,13 +1025,13 @@
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>9.537933765391532e-12</v>
+        <v>-1.929097524979682e-13</v>
       </c>
       <c r="F8" t="n">
-        <v>-1.895739451098215e-12</v>
+        <v>-1.570266536619102e-13</v>
       </c>
       <c r="G8" t="n">
-        <v>4.049249829109179e-12</v>
+        <v>3.278131402773022e-14</v>
       </c>
     </row>
     <row r="9">
@@ -1054,13 +1054,13 @@
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>-2.651270564303874e-12</v>
+        <v>-3.846776083034307e-13</v>
       </c>
       <c r="F9" t="n">
-        <v>-1.260972030742751e-11</v>
+        <v>-1.305457196455309e-13</v>
       </c>
       <c r="G9" t="n">
-        <v>3.68584273497127e-12</v>
+        <v>5.063041270366415e-14</v>
       </c>
     </row>
     <row r="10">
@@ -1083,13 +1083,13 @@
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>-1.351501105190982e-11</v>
+        <v>-4.637209456844224e-13</v>
       </c>
       <c r="F10" t="n">
-        <v>-1.697453936285641e-11</v>
+        <v>-2.564010832324607e-13</v>
       </c>
       <c r="G10" t="n">
-        <v>1.667643442237405e-12</v>
+        <v>1.057915193878415e-14</v>
       </c>
     </row>
     <row r="11">
@@ -1112,13 +1112,13 @@
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>-8.012161980540217e-12</v>
+        <v>4.396979844506709e-13</v>
       </c>
       <c r="F11" t="n">
-        <v>-6.451795657549519e-12</v>
+        <v>1.343228642793301e-13</v>
       </c>
       <c r="G11" t="n">
-        <v>-7.74519215365475e-12</v>
+        <v>-1.057011731129185e-13</v>
       </c>
     </row>
     <row r="12">
@@ -1141,13 +1141,13 @@
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>1.786962596488065e-11</v>
+        <v>-4.562420158107729e-13</v>
       </c>
       <c r="F12" t="n">
-        <v>7.851994324196461e-12</v>
+        <v>-1.412789767697908e-13</v>
       </c>
       <c r="G12" t="n">
-        <v>-7.742587541601068e-12</v>
+        <v>-2.470862036551376e-13</v>
       </c>
     </row>
     <row r="13">
@@ -1170,13 +1170,13 @@
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>-1.586262827861592e-11</v>
+        <v>-4.605521514763177e-13</v>
       </c>
       <c r="F13" t="n">
-        <v>-9.827480519235354e-12</v>
+        <v>3.652724404823173e-14</v>
       </c>
       <c r="G13" t="n">
-        <v>-1.286750195291898e-11</v>
+        <v>-2.384121443557254e-13</v>
       </c>
     </row>
     <row r="14">
@@ -1196,16 +1196,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-1.452802856018534e-11</v>
+        <v>-4.240562490976821e-13</v>
       </c>
       <c r="E14" t="n">
         <v/>
       </c>
       <c r="F14" t="n">
-        <v>-1.168183917568195e-11</v>
+        <v>3.556946311808718e-14</v>
       </c>
       <c r="G14" t="n">
-        <v>-2.864535584489709e-12</v>
+        <v>7.663896634290298e-15</v>
       </c>
     </row>
     <row r="15">
@@ -1225,16 +1225,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-1.427450810858471e-11</v>
+        <v>-4.743580066259649e-13</v>
       </c>
       <c r="E15" t="n">
         <v/>
       </c>
       <c r="F15" t="n">
-        <v>-3.624002262349633e-12</v>
+        <v>4.93622801201245e-14</v>
       </c>
       <c r="G15" t="n">
-        <v>1.485620989102121e-11</v>
+        <v>6.62869096027434e-12</v>
       </c>
     </row>
     <row r="16">
@@ -1254,16 +1254,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-1.793102768287622e-11</v>
+        <v>-4.687987140472853e-13</v>
       </c>
       <c r="E16" t="n">
         <v/>
       </c>
       <c r="F16" t="n">
-        <v>-1.627524578555356e-11</v>
+        <v>-9.540355736118977e-15</v>
       </c>
       <c r="G16" t="n">
-        <v>1.817371705788239e-11</v>
+        <v>3.457370194128334e-11</v>
       </c>
     </row>
     <row r="17">
@@ -1283,16 +1283,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5.976818521884822e-11</v>
+        <v>3.230372998103911e-10</v>
       </c>
       <c r="E17" t="n">
         <v/>
       </c>
       <c r="F17" t="n">
-        <v>-5.441786387527748e-12</v>
+        <v>2.388154776122449e-13</v>
       </c>
       <c r="G17" t="n">
-        <v>1.728036528730651e-11</v>
+        <v>2.582677743071036e-11</v>
       </c>
     </row>
     <row r="18">
@@ -1312,16 +1312,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5.400149010303645e-12</v>
+        <v>9.006337579644005e-13</v>
       </c>
       <c r="E18" t="n">
         <v/>
       </c>
       <c r="F18" t="n">
-        <v>1.597656021489842e-11</v>
+        <v>2.228073351849644e-12</v>
       </c>
       <c r="G18" t="n">
-        <v>1.956375752664949e-11</v>
+        <v>1.702631996145832e-11</v>
       </c>
     </row>
     <row r="19">
@@ -1341,16 +1341,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4.023547659661556e-11</v>
+        <v>-3.930397357214853e-13</v>
       </c>
       <c r="E19" t="n">
         <v/>
       </c>
       <c r="F19" t="n">
-        <v>3.127109109756888e-11</v>
+        <v>5.423308406397197e-14</v>
       </c>
       <c r="G19" t="n">
-        <v>0.08771334602754001</v>
+        <v>0.2344115891459782</v>
       </c>
     </row>
     <row r="20">
@@ -1370,16 +1370,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2.425473771030531e-12</v>
+        <v>-4.018457084810005e-13</v>
       </c>
       <c r="E20" t="n">
         <v/>
       </c>
       <c r="F20" t="n">
-        <v>-1.170329866226097e-11</v>
+        <v>-1.425156208628865e-13</v>
       </c>
       <c r="G20" t="n">
-        <v>1.508254487474385e-11</v>
+        <v>9.436661632932083e-12</v>
       </c>
     </row>
     <row r="21">
@@ -1399,16 +1399,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-8.384283938830536e-12</v>
+        <v>6.239255888635602e-13</v>
       </c>
       <c r="E21" t="n">
         <v/>
       </c>
       <c r="F21" t="n">
-        <v>-1.071485406460949e-11</v>
+        <v>5.584719408712585e-14</v>
       </c>
       <c r="G21" t="n">
-        <v>-1.430471476492712e-12</v>
+        <v>2.782719140479434e-14</v>
       </c>
     </row>
     <row r="22">
@@ -1428,16 +1428,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-1.603391868979762e-11</v>
+        <v>-4.653678363918718e-13</v>
       </c>
       <c r="E22" t="n">
         <v/>
       </c>
       <c r="F22" t="n">
-        <v>-1.670564905891367e-11</v>
+        <v>-1.718636193271544e-13</v>
       </c>
       <c r="G22" t="n">
-        <v>1.885654539389515e-11</v>
+        <v>1.827128055358961e-11</v>
       </c>
     </row>
     <row r="23">
@@ -1457,16 +1457,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-3.894335529836792e-12</v>
+        <v>-4.443679433585124e-13</v>
       </c>
       <c r="E23" t="n">
         <v/>
       </c>
       <c r="F23" t="n">
-        <v>-1.437762437622417e-11</v>
+        <v>-2.058852723812102e-14</v>
       </c>
       <c r="G23" t="n">
-        <v>-2.06031087272237e-12</v>
+        <v>5.94661773457934e-12</v>
       </c>
     </row>
     <row r="24">
@@ -1486,16 +1486,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2.295465314275205e-11</v>
+        <v>-4.23600645579187e-13</v>
       </c>
       <c r="E24" t="n">
         <v/>
       </c>
       <c r="F24" t="n">
-        <v>2.246422111767813e-11</v>
+        <v>-7.211909808888959e-14</v>
       </c>
       <c r="G24" t="n">
-        <v>4.592470064151585e-12</v>
+        <v>-1.252286894128361e-14</v>
       </c>
     </row>
     <row r="25">
@@ -1515,16 +1515,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>-1.296666943765017e-11</v>
+        <v>-4.698257571619757e-13</v>
       </c>
       <c r="E25" t="n">
         <v/>
       </c>
       <c r="F25" t="n">
-        <v>-9.917321764434639e-12</v>
+        <v>-2.859145010982665e-14</v>
       </c>
       <c r="G25" t="n">
-        <v>-1.824076274651307e-12</v>
+        <v>4.08075845618547e-12</v>
       </c>
     </row>
     <row r="26">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-1.521758002512574e-11</v>
+        <v>-2.273794888442601e-13</v>
       </c>
       <c r="E26" t="n">
-        <v>-1.083197062852224e-11</v>
+        <v>7.163653175567448e-14</v>
       </c>
       <c r="F26" t="n">
         <v/>
       </c>
       <c r="G26" t="n">
-        <v>-2.939048477406122e-12</v>
+        <v>9.717777207300968e-11</v>
       </c>
     </row>
     <row r="27">
@@ -1573,16 +1573,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-5.965153093173938e-12</v>
+        <v>-1.916336113948813e-13</v>
       </c>
       <c r="E27" t="n">
-        <v>4.593774577486427e-12</v>
+        <v>-5.088387553137106e-15</v>
       </c>
       <c r="F27" t="n">
         <v/>
       </c>
       <c r="G27" t="n">
-        <v>-2.900888553334803e-13</v>
+        <v>3.264130070697264e-15</v>
       </c>
     </row>
     <row r="28">
@@ -1602,16 +1602,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-1.75162956302478e-11</v>
+        <v>-1.903692564551217e-13</v>
       </c>
       <c r="E28" t="n">
-        <v>-1.527907662514424e-11</v>
+        <v>-2.333716114913557e-14</v>
       </c>
       <c r="F28" t="n">
         <v/>
       </c>
       <c r="G28" t="n">
-        <v>3.179249091760918e-11</v>
+        <v>4.577000305025418e-10</v>
       </c>
     </row>
     <row r="29">
@@ -1631,16 +1631,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.004588699972024e-12</v>
+        <v>3.750123575404834e-13</v>
       </c>
       <c r="E29" t="n">
-        <v>-1.272032191893727e-11</v>
+        <v>-1.127373364706171e-13</v>
       </c>
       <c r="F29" t="n">
         <v/>
       </c>
       <c r="G29" t="n">
-        <v>2.051953414842449e-12</v>
+        <v>1.890002835025863e-10</v>
       </c>
     </row>
     <row r="30">
@@ -1660,16 +1660,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.360039941945333e-11</v>
+        <v>3.219048200009372e-13</v>
       </c>
       <c r="E30" t="n">
-        <v>4.743550827787758e-12</v>
+        <v>8.19078256974344e-14</v>
       </c>
       <c r="F30" t="n">
         <v/>
       </c>
       <c r="G30" t="n">
-        <v>1.314610145403371e-11</v>
+        <v>8.866880388515548e-15</v>
       </c>
     </row>
     <row r="31">
@@ -1689,16 +1689,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.09407729251698e-11</v>
+        <v>-1.140909165197949e-13</v>
       </c>
       <c r="E31" t="n">
-        <v>6.401815555301483e-12</v>
+        <v>-1.740188374639116e-13</v>
       </c>
       <c r="F31" t="n">
         <v/>
       </c>
       <c r="G31" t="n">
-        <v>4.79963629215062e-11</v>
+        <v>3.591404185347176e-10</v>
       </c>
     </row>
     <row r="32">
@@ -1718,16 +1718,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>-2.396899927610364e-11</v>
+        <v>3.968387531245985e-12</v>
       </c>
       <c r="E32" t="n">
-        <v>7.644607336737013e-12</v>
+        <v>1.773661240606442e-13</v>
       </c>
       <c r="F32" t="n">
         <v/>
       </c>
       <c r="G32" t="n">
-        <v>3.785072747688351e-11</v>
+        <v>2.921232329711815e-10</v>
       </c>
     </row>
     <row r="33">
@@ -1747,16 +1747,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3.279704807997617e-11</v>
+        <v>9.95916205384478e-13</v>
       </c>
       <c r="E33" t="n">
-        <v>2.758008292905682e-11</v>
+        <v>2.207727637101358e-12</v>
       </c>
       <c r="F33" t="n">
         <v/>
       </c>
       <c r="G33" t="n">
-        <v>7.800522718524912e-11</v>
+        <v>3.911908613071968e-10</v>
       </c>
     </row>
     <row r="34">
@@ -1776,16 +1776,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-2.695699462934695e-12</v>
+        <v>2.09124533026004e-13</v>
       </c>
       <c r="E34" t="n">
-        <v>-5.863831572424522e-12</v>
+        <v>6.753110390431823e-14</v>
       </c>
       <c r="F34" t="n">
         <v/>
       </c>
       <c r="G34" t="n">
-        <v>-6.913298536712035e-12</v>
+        <v>0.000930298149127694</v>
       </c>
     </row>
     <row r="35">
@@ -1805,16 +1805,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>-9.678516615905695e-12</v>
+        <v>2.208903528840282e-13</v>
       </c>
       <c r="E35" t="n">
-        <v>-1.624922906266346e-11</v>
+        <v>-1.93435507715525e-14</v>
       </c>
       <c r="F35" t="n">
         <v/>
       </c>
       <c r="G35" t="n">
-        <v>-1.122028328023902e-11</v>
+        <v>7.375755023185555e-11</v>
       </c>
     </row>
     <row r="36">
@@ -1834,16 +1834,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8.116632788080704e-12</v>
+        <v>-1.928094321323713e-13</v>
       </c>
       <c r="E36" t="n">
-        <v>1.111730283949088e-11</v>
+        <v>-4.630719902947737e-14</v>
       </c>
       <c r="F36" t="n">
         <v/>
       </c>
       <c r="G36" t="n">
-        <v>-1.187176091811423e-11</v>
+        <v>5.978093553748223e-11</v>
       </c>
     </row>
     <row r="37">
@@ -1863,16 +1863,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>-7.639222783137163e-12</v>
+        <v>-1.206488595288371e-13</v>
       </c>
       <c r="E37" t="n">
-        <v>-9.44257794864357e-12</v>
+        <v>-6.369812058088295e-14</v>
       </c>
       <c r="F37" t="n">
         <v/>
       </c>
       <c r="G37" t="n">
-        <v>-1.246517049493312e-11</v>
+        <v>5.511866263670527e-16</v>
       </c>
     </row>
     <row r="38">
@@ -1892,13 +1892,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-1.026801716732619e-11</v>
+        <v>-1.93396766704574e-13</v>
       </c>
       <c r="E38" t="n">
-        <v>2.235072289236996e-11</v>
+        <v>1.990743609245712e-11</v>
       </c>
       <c r="F38" t="n">
-        <v>-1.886513315332456e-12</v>
+        <v>1.435782316428451e-10</v>
       </c>
       <c r="G38" t="n">
         <v/>
@@ -1921,13 +1921,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-9.822812318639854e-12</v>
+        <v>-2.099622147273987e-13</v>
       </c>
       <c r="E39" t="n">
-        <v>1.454460336916533e-11</v>
+        <v>6.436042753398332e-12</v>
       </c>
       <c r="F39" t="n">
-        <v>1.965523636074852e-11</v>
+        <v>3.373464703998906e-10</v>
       </c>
       <c r="G39" t="n">
         <v/>
@@ -1950,13 +1950,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-6.91511282149352e-12</v>
+        <v>1.612926376757452e-14</v>
       </c>
       <c r="E40" t="n">
-        <v>-5.583020673873377e-12</v>
+        <v>2.237275070074182e-14</v>
       </c>
       <c r="F40" t="n">
-        <v>6.704819144748515e-12</v>
+        <v>4.554416641709056e-15</v>
       </c>
       <c r="G40" t="n">
         <v/>
@@ -1979,13 +1979,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>8.976036598790981e-12</v>
+        <v>-2.688588180508932e-15</v>
       </c>
       <c r="E41" t="n">
-        <v>6.980303643901265e-12</v>
+        <v>3.88739129481063e-12</v>
       </c>
       <c r="F41" t="n">
-        <v>-4.86868326915172e-12</v>
+        <v>1.140558957401734e-10</v>
       </c>
       <c r="G41" t="n">
         <v/>
@@ -2008,13 +2008,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2.280826826604378e-12</v>
+        <v>2.801852342770348e-15</v>
       </c>
       <c r="E42" t="n">
-        <v>9.071088603446623e-12</v>
+        <v>4.6529069099372e-12</v>
       </c>
       <c r="F42" t="n">
-        <v>4.533606668684886e-11</v>
+        <v>4.102517862589867e-10</v>
       </c>
       <c r="G42" t="n">
         <v/>
@@ -2037,13 +2037,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1.152972352701211e-11</v>
+        <v>-1.683423813482911e-14</v>
       </c>
       <c r="E43" t="n">
-        <v>1.11628191054395e-11</v>
+        <v>-8.634588360272093e-15</v>
       </c>
       <c r="F43" t="n">
-        <v>3.564415473149497e-12</v>
+        <v>6.993833914999635e-15</v>
       </c>
       <c r="G43" t="n">
         <v/>
@@ -2066,13 +2066,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>4.669711236471972e-12</v>
+        <v>-3.542028557484691e-14</v>
       </c>
       <c r="E44" t="n">
-        <v>1.329740068311387e-11</v>
+        <v>4.771695118446148e-12</v>
       </c>
       <c r="F44" t="n">
-        <v>-1.185647016475671e-11</v>
+        <v>3.308923550887533e-11</v>
       </c>
       <c r="G44" t="n">
         <v/>
@@ -2095,13 +2095,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>-1.18963846717152e-12</v>
+        <v>1.477467529562202e-14</v>
       </c>
       <c r="E45" t="n">
-        <v>2.799577804116261e-11</v>
+        <v>1.740734312445986e-11</v>
       </c>
       <c r="F45" t="n">
-        <v>-7.490936572785843e-12</v>
+        <v>3.903687925388278e-11</v>
       </c>
       <c r="G45" t="n">
         <v/>
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>-4.576316438838688e-12</v>
+        <v>1.501295702358367e-14</v>
       </c>
       <c r="E46" t="n">
-        <v>-5.53996709329746e-12</v>
+        <v>6.7638995979212e-15</v>
       </c>
       <c r="F46" t="n">
-        <v>-1.00674229526002e-11</v>
+        <v>-3.860308565945727e-16</v>
       </c>
       <c r="G46" t="n">
         <v/>
@@ -2153,13 +2153,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-8.502622405788954e-12</v>
+        <v>4.440460364958887e-12</v>
       </c>
       <c r="E47" t="n">
-        <v>1.110330137155522e-11</v>
+        <v>1.770676518331062e-11</v>
       </c>
       <c r="F47" t="n">
-        <v>4.139321891188414e-11</v>
+        <v>3.337841252103346e-10</v>
       </c>
       <c r="G47" t="n">
         <v/>
@@ -2182,13 +2182,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3.428734793144072e-11</v>
+        <v>1.644864751661527e-13</v>
       </c>
       <c r="E48" t="n">
-        <v>0.08680781078633565</v>
+        <v>0.2319915694869344</v>
       </c>
       <c r="F48" t="n">
-        <v>5.340924877920914e-11</v>
+        <v>3.416995649363569e-10</v>
       </c>
       <c r="G48" t="n">
         <v/>
@@ -2211,13 +2211,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6.511003284236637e-12</v>
+        <v>2.013769975936149e-13</v>
       </c>
       <c r="E49" t="n">
-        <v>1.215803704431304e-11</v>
+        <v>1.10968524791923e-11</v>
       </c>
       <c r="F49" t="n">
-        <v>-6.957592901068361e-12</v>
+        <v>0.00092228784102166</v>
       </c>
       <c r="G49" t="n">
         <v/>
@@ -2239,7 +2239,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>0.009943354874849319</v>
+        <v>0.01249032653868198</v>
       </c>
     </row>
   </sheetData>
@@ -2283,7 +2283,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.2497696535404925</v>
+        <v>0.6675464642582738</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -2308,7 +2308,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>3.103255151979978e-09</v>
+        <v>9.946752740721716e-05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>